<commit_message>
site build 2026-10-08 21:01
</commit_message>
<xml_diff>
--- a/models/sovereigns/Albania_Sovereign_Model.xlsx
+++ b/models/sovereigns/Albania_Sovereign_Model.xlsx
@@ -637,16 +637,34 @@
           <t>policy_rate_pct</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
+      <c r="B3" s="2" t="n">
+        <v>2.5</v>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>IMF MFS interest rates</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>IMF MFS interest rates, monetary policy-related rate, % p.a., monthly (auto-filled; a run's sourced point replaces it unless older)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -671,16 +689,34 @@
           <t>cpi_latest_yoy_pct</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n"/>
+      <c r="B5" s="2" t="n">
+        <v>3.3508</v>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>IMF CPI database</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>IMF CPI database, all items, y/y % change, monthly (auto-filled; a run's sourced point replaces it unless older)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -755,7 +791,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO via database/sovereigns/albania.json</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -765,7 +801,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
+          <t>General government debt, IMF WEO; vintage not stated</t>
         </is>
       </c>
     </row>
@@ -949,7 +985,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>8.602</v>
+        <v>9.347</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -958,12 +994,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>World Bank WDI</t>
+          <t>IMF International Liquidity</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -973,7 +1009,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
+          <t>Gross official reserves incl. gold at national valuation, end-month (auto-filled; a run's sourced point replaces it unless older)</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1037,7 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>7.208</v>
+        <v>7.2</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1015,7 +1051,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>World Bank WDI</t>
+          <t>World Bank via database/sovereigns/albania.json</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1023,11 +1059,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1052,16 +1084,34 @@
           <t>external_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n"/>
+      <c r="B20" s="2" t="n">
+        <v>39.7</v>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>% GDP</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>World Bank via database/sovereigns/albania.json</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>External debt as % of GNI (World Bank), not GDP</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1087,7 +1137,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>33.333</v>
+        <v>33.3</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1101,7 +1151,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO via database/sovereigns/albania.json</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1109,11 +1159,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1244,7 +1290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1258,6 +1304,31 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
@@ -1268,7 +1339,18 @@
           <t>nominal_gdp_usd_bn</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1276,7 +1358,12 @@
           <t>real_gdp_growth_pct</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1284,7 +1371,12 @@
           <t>cpi_avg_pct</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1292,7 +1384,12 @@
           <t>current_account_pct_gdp</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1300,7 +1397,12 @@
           <t>fiscal_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1308,7 +1410,12 @@
           <t>primary_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1316,7 +1423,26 @@
           <t>gov_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" s="2" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1324,7 +1450,20 @@
           <t>external_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" s="2" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>World Bank (% of GNI) via database/sovereigns/albania.json, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1332,7 +1471,18 @@
           <t>gross_reserves_usd_bn</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>World Bank via database/sovereigns/albania.json, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1340,7 +1490,12 @@
           <t>revenue_pct_gdp</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1348,7 +1503,12 @@
           <t>interest_pct_revenue</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
site build 2026-10-09 06:57
</commit_message>
<xml_diff>
--- a/models/sovereigns/Albania_Sovereign_Model.xlsx
+++ b/models/sovereigns/Albania_Sovereign_Model.xlsx
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 08-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/albania.json</t>
+          <t>built 09-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/albania.json</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>9.347</v>
+        <v>8.6</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -994,12 +994,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>IMF International Liquidity</t>
+          <t>World Bank via database/sovereigns/albania.json</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Gross official reserves incl. gold at national valuation, end-month (auto-filled; a run's sourced point replaces it unless older)</t>
+          <t>as reported by World Bank via repo file; gold inclusion not stated</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>External debt as % of GNI (World Bank), not GDP</t>
+          <t>External debt stock as % of GNI (not GDP), World Bank</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-09 07:19
</commit_message>
<xml_diff>
--- a/models/sovereigns/Albania_Sovereign_Model.xlsx
+++ b/models/sovereigns/Albania_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 08-Oct-26</t>
+          <t>as of 09-Oct-26</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json</t>
+          <t>IMF WEO via database/sovereigns/albania.json (vintage not stated)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>General government debt, IMF WEO; vintage not stated</t>
+          <t>general government debt</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>as reported by World Bank via repo file; gold inclusion not stated</t>
+          <t>gross FX reserves per World Bank series; gold treatment not stated</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>External debt stock as % of GNI (not GDP), World Bank</t>
+          <t>external debt as % of GNI (World Bank), not % of GDP</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json</t>
+          <t>IMF WEO via database/sovereigns/albania.json (vintage not stated)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26</t>
+          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26 (general government debt; vintage not stated)</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       <c r="F9" s="2" t="n"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>World Bank (% of GNI) via database/sovereigns/albania.json, 08-Oct-26</t>
+          <t>World Bank via database/sovereigns/albania.json, 08-Oct-26 (% of GNI)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-09 08:09
</commit_message>
<xml_diff>
--- a/models/sovereigns/Albania_Sovereign_Model.xlsx
+++ b/models/sovereigns/Albania_Sovereign_Model.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json (vintage not stated)</t>
+          <t>IMF WEO via database/sovereigns/albania.json</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross FX reserves per World Bank series; gold treatment not stated</t>
+          <t>gross FX reserves, World Bank definition (gold treatment not stated)</t>
         </is>
       </c>
     </row>
@@ -1067,16 +1067,34 @@
           <t>short_term_external_debt_usd_bn</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n"/>
+      <c r="B19" s="2" t="n">
+        <v>1.63</v>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>USD bn</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>World Bank via database/sovereigns/albania.json</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>19.0% of gross reserves of $8.60bn (derived)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1109,7 +1127,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>external debt as % of GNI (World Bank), not % of GDP</t>
+          <t>external debt as % of GNI (not GDP), World Bank</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1169,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json (vintage not stated)</t>
+          <t>IMF WEO via database/sovereigns/albania.json</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1440,7 +1458,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26 (general government debt; vintage not stated)</t>
+          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26 (vintage not stated)</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1479,7 @@
       <c r="F9" s="2" t="n"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>World Bank via database/sovereigns/albania.json, 08-Oct-26 (% of GNI)</t>
+          <t>World Bank (% of GNI, not GDP) via database/sovereigns/albania.json, 08-Oct-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-09 08:13
</commit_message>
<xml_diff>
--- a/models/sovereigns/Albania_Sovereign_Model.xlsx
+++ b/models/sovereigns/Albania_Sovereign_Model.xlsx
@@ -801,7 +801,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>general government debt</t>
+          <t>General government debt, IMF WEO; vintage not stated</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross FX reserves, World Bank definition (gold treatment not stated)</t>
+          <t>as stated by World Bank; inclusion of gold not stated</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26 (vintage not stated)</t>
+          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-09 09:09
</commit_message>
<xml_diff>
--- a/models/sovereigns/Albania_Sovereign_Model.xlsx
+++ b/models/sovereigns/Albania_Sovereign_Model.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json</t>
+          <t>IMF WEO via database/sovereigns/albania.json (vintage not stated)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>General government debt, IMF WEO; vintage not stated</t>
+          <t>general government debt, IMF WEO</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>as stated by World Bank; inclusion of gold not stated</t>
+          <t>gross FX reserves as reported by World Bank; gold treatment not stated</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>external debt as % of GNI (not GDP), World Bank</t>
+          <t>external debt as % of GNI (World Bank), not % of GDP</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json</t>
+          <t>IMF WEO via database/sovereigns/albania.json (vintage not stated)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26</t>
+          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26 (vintage not stated)</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
       <c r="F9" s="2" t="n"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>World Bank (% of GNI, not GDP) via database/sovereigns/albania.json, 08-Oct-26</t>
+          <t>World Bank via database/sovereigns/albania.json, 08-Oct-26 (% of GNI, not GDP)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-10 05:19
</commit_message>
<xml_diff>
--- a/models/sovereigns/Albania_Sovereign_Model.xlsx
+++ b/models/sovereigns/Albania_Sovereign_Model.xlsx
@@ -801,7 +801,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>general government debt, IMF WEO</t>
+          <t>General government debt</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross FX reserves as reported by World Bank; gold treatment not stated</t>
+          <t>as reported by World Bank via repo file; gold inclusion not stated</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>external debt as % of GNI (World Bank), not % of GDP</t>
+          <t>External debt as % of GNI (World Bank), not % of GDP</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26 (vintage not stated)</t>
+          <t>IMF WEO via database/sovereigns/albania.json, 08-Oct-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-19 07:30
</commit_message>
<xml_diff>
--- a/models/sovereigns/Albania_Sovereign_Model.xlsx
+++ b/models/sovereigns/Albania_Sovereign_Model.xlsx
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 12-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/albania.json</t>
+          <t>built 19-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/albania.json</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>19-Oct-26</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>19-Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>8.6</v>
+        <v>9.347</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -994,22 +994,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>World Bank via database/sovereigns/albania.json</t>
+          <t>IMF International Liquidity</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>19-Oct-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>as reported by World Bank via repo file; gold inclusion not stated</t>
+          <t>Gross official reserves incl. gold at national valuation, end-month (auto-filled; a run's sourced point replaces it unless older)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-26 07:30
</commit_message>
<xml_diff>
--- a/models/sovereigns/Albania_Sovereign_Model.xlsx
+++ b/models/sovereigns/Albania_Sovereign_Model.xlsx
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 19-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/albania.json</t>
+          <t>built 26-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/albania.json</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>19-Oct-26</t>
+          <t>26-Oct-26</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>19-Oct-26</t>
+          <t>26-Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>9.347</v>
+        <v>9.756</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>19-Oct-26</t>
+          <t>26-Oct-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">

</xml_diff>